<commit_message>
Liga cada usuário a um responsável, mostra agendamentos no Calendário e edita a safra
- Usuário passa a ter nomeResponsavel (Admin → Usuários); usuário comum só altera os clientes
  dele, e qualquer um agenda (regras em lib/responsavel.ts, com testes)
- Cliente ganha o campo comercial (cadastro, importação da planilha e equipe por região)
- Agendamento registra quem agendou e quando (agendadoPor/agendadoEm)
- Calendário mostra os agendamentos da safra com legenda por status; atividades só podem ser
  alteradas pelo dono ou por um admin
- Admin → Safras edita nome, cultura e período; título do Pré-Safra segue a safra selecionada
- Novo cliente: usuário comum fica como responsável e o admin escolhe o comercial
- Painel passa a ser aberto a todos os usuários (somente leitura)

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/modelo-importacao-clientes.xlsx
+++ b/public/modelo-importacao-clientes.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="22">
   <si>
     <t>Cliente</t>
   </si>
@@ -31,6 +31,9 @@
     <t>Consultor</t>
   </si>
   <si>
+    <t>Comercial</t>
+  </si>
+  <si>
     <t>Agrícola Grão de Ouro</t>
   </si>
   <si>
@@ -47,6 +50,9 @@
   </si>
   <si>
     <t>Carlos Souza</t>
+  </si>
+  <si>
+    <t>Sidinei</t>
   </si>
   <si>
     <t>Fazenda Boa Vista</t>
@@ -451,17 +457,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
     <col min="3" max="3" width="8" customWidth="1"/>
     <col min="4" max="4" width="28" customWidth="1"/>
-    <col min="5" max="6" width="22" customWidth="1"/>
+    <col min="5" max="7" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -480,69 +486,78 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F2" t="s">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="G2" t="s">
+        <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G3" t="s">
         <v>13</v>
-      </c>
-      <c r="C3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E3" t="s">
-        <v>16</v>
-      </c>
-      <c r="F3" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B4" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C4" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D4" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E4" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F4" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>